<commit_message>
run experiments e relatorio
</commit_message>
<xml_diff>
--- a/trabGramos/outputs/tables/nn_best3.xlsx
+++ b/trabGramos/outputs/tables/nn_best3.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="81" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="108" uniqueCount="30">
   <si>
     <t>config_name</t>
   </si>
@@ -79,6 +79,30 @@
   </si>
   <si>
     <t>outputs\nn\best_nn_10_trainscg_60_20_20_raw.mat</t>
+  </si>
+  <si>
+    <t>nn_10_trainscg_70_15_15_raw</t>
+  </si>
+  <si>
+    <t>nn_10_trainscg_70_15_15_norm</t>
+  </si>
+  <si>
+    <t>nn_10_traingdx_70_15_15_raw</t>
+  </si>
+  <si>
+    <t>traingdx</t>
+  </si>
+  <si>
+    <t>[0.7 0.15 0.15]</t>
+  </si>
+  <si>
+    <t>outputs\nn\best_nn_10_trainscg_70_15_15_raw.mat</t>
+  </si>
+  <si>
+    <t>outputs\nn\best_nn_10_trainscg_70_15_15_norm.mat</t>
+  </si>
+  <si>
+    <t>outputs\nn\best_nn_10_traingdx_70_15_15_raw.mat</t>
   </si>
 </sst>
 </file>
@@ -127,10 +151,10 @@
   <dimension ref="A1:L4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="27.36328125" customWidth="true"/>
+    <col min="1" max="1" width="28.08984375" customWidth="true"/>
     <col min="2" max="2" width="12.6328125" customWidth="true"/>
     <col min="3" max="3" width="8.36328125" customWidth="true"/>
-    <col min="4" max="4" width="11.6328125" customWidth="true"/>
+    <col min="4" max="4" width="12.7265625" customWidth="true"/>
     <col min="5" max="5" width="15.36328125" customWidth="true"/>
     <col min="6" max="6" width="12" customWidth="true"/>
     <col min="7" max="7" width="19.81640625" customWidth="true"/>
@@ -138,7 +162,7 @@
     <col min="9" max="9" width="17.90625" customWidth="true"/>
     <col min="10" max="10" width="15.7265625" customWidth="true"/>
     <col min="11" max="11" width="8.26953125" customWidth="true"/>
-    <col min="12" max="12" width="46" customWidth="true"/>
+    <col min="12" max="12" width="46.7265625" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -181,116 +205,116 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="B2" s="0" t="s">
         <v>5</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="E2" s="0" t="b">
         <v>0</v>
       </c>
       <c r="F2" s="0">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G2" s="0">
-        <v>99.980000000000004</v>
+        <v>99.978000000000023</v>
       </c>
       <c r="H2" s="0">
-        <v>0</v>
+        <v>0.019888578520234124</v>
       </c>
       <c r="I2" s="0">
-        <v>99.900000000000006</v>
+        <v>99.960000000000008</v>
       </c>
       <c r="J2" s="0">
-        <v>0</v>
+        <v>0.0644061188719494</v>
       </c>
       <c r="K2" s="0">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L2" s="0" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="B3" s="0" t="s">
         <v>5</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="E3" s="0" t="b">
         <v>1</v>
       </c>
       <c r="F3" s="0">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G3" s="0">
-        <v>99.980000000000004</v>
+        <v>99.978000000000023</v>
       </c>
       <c r="H3" s="0">
-        <v>0</v>
+        <v>0.019888578520234124</v>
       </c>
       <c r="I3" s="0">
-        <v>99.900000000000006</v>
+        <v>99.960000000000008</v>
       </c>
       <c r="J3" s="0">
-        <v>0</v>
+        <v>0.0644061188719494</v>
       </c>
       <c r="K3" s="0">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L3" s="0" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="B4" s="0" t="s">
         <v>5</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="E4" s="0" t="b">
         <v>0</v>
       </c>
       <c r="F4" s="0">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G4" s="0">
-        <v>99.980000000000004</v>
+        <v>99.975999999999999</v>
       </c>
       <c r="H4" s="0">
-        <v>0</v>
+        <v>0.022705848487902358</v>
       </c>
       <c r="I4" s="0">
-        <v>99.900000000000006</v>
+        <v>99.960000000000008</v>
       </c>
       <c r="J4" s="0">
-        <v>0</v>
+        <v>0.0644061188719494</v>
       </c>
       <c r="K4" s="0">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L4" s="0" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>